<commit_message>
fix: unify lab weights across same-list groups
21 groups, 36 sheets. Reference BWCCI > WEAB > BMET > BGMEA.
WEAB + BWCCI-Residential Fashion Design rebuilt from BWCCI (19 items).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01EYF8ZViZ52j72cGLCGYpbD
</commit_message>
<xml_diff>
--- a/data/xlsx/aeosib--marine-engine-operation-and-maintenance.xlsx
+++ b/data/xlsx/aeosib--marine-engine-operation-and-maintenance.xlsx
@@ -702,7 +702,7 @@
         <v>0</v>
       </c>
       <c r="E19" s="27" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F19" s="27">
         <f>IFERROR(MIN(C19,D19)*E19/C19,0)</f>
@@ -726,7 +726,7 @@
         <v>0</v>
       </c>
       <c r="E20" s="27" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F20" s="27">
         <f>IFERROR(MIN(C20,D20)*E20/C20,0)</f>
@@ -774,7 +774,7 @@
         <v>0</v>
       </c>
       <c r="E22" s="27" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F22" s="27">
         <f>IFERROR(MIN(C22,D22)*E22/C22,0)</f>
@@ -846,7 +846,7 @@
         <v>0</v>
       </c>
       <c r="E25" s="27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F25" s="27">
         <f>IFERROR(MIN(C25,D25)*E25/C25,0)</f>
@@ -870,7 +870,7 @@
         <v>0</v>
       </c>
       <c r="E26" s="27" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F26" s="27">
         <f>IFERROR(MIN(C26,D26)*E26/C26,0)</f>
@@ -894,7 +894,7 @@
         <v>0</v>
       </c>
       <c r="E27" s="27" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="F27" s="27">
         <f>IFERROR(MIN(C27,D27)*E27/C27,0)</f>

</xml_diff>